<commit_message>
Update daily stock monitor reports
</commit_message>
<xml_diff>
--- a/data/BOLL/EXCLE/AMD_1_20260826.xlsx
+++ b/data/BOLL/EXCLE/AMD_1_20260826.xlsx
@@ -196,12 +196,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'30日跟踪'!$A$8</f>
+              <f>'30日跟踪'!$A$8:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'30日跟踪'!$D$8</f>
+              <f>'30日跟踪'!$D$8:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
     </row>
     <row r="6">
@@ -660,7 +660,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1/30</t>
+          <t>2/30</t>
         </is>
       </c>
     </row>
@@ -708,6 +708,26 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>第1/30个交易日</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>476.6700134277344</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>-0.8857794924257756</v>
+      </c>
+      <c r="D9" s="6">
+        <f>B9/$B$8-1</f>
+        <v/>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>第2/30个交易日</t>
         </is>
       </c>
     </row>

</xml_diff>